<commit_message>
Translate 'Top' button label into all 11 languages
Add top_btn key to all language blocks; wire to <span data-i18n="top_btn"> in scroll-to-top button; update all 8 translation spreadsheets.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B160"/>
+  <dimension ref="A1:B161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55.83203125" customWidth="1" min="1" max="1"/>
@@ -2377,6 +2377,18 @@
         </is>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Oben</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update translation spreadsheets: add kofi_btn_label (Buy me a coffee) row 162
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B161"/>
+  <dimension ref="A1:B162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55.83203125" customWidth="1" min="1" max="1"/>
@@ -2389,6 +2389,18 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Buy me a coffee</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Kauf mir einen Kaffee</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update translation spreadsheets with cgats_header_warning (row 163)
All 8 Eng-*.xlsx files updated from 162 to 163 rows.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B162"/>
+  <dimension ref="A1:B163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55.83203125" customWidth="1" min="1" max="1"/>
@@ -2401,6 +2401,18 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>File header is not standard CGATS (first line does not contain “CGATS” or “ISO28178”)</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Dateikopfzeile entspricht nicht Standard-CGATS (erste Zeile enthält weder „CGATS“ noch „ISO28178“)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Swedish language; fix Chinese gain translation; update translation spreadsheets
- Add Swedish (sv) as a new UI language with full translation
- Fix zh-CN and zh-TW: gain '增益' → '增大' (consistent with tone_value_gain)
- Rebuild all translation spreadsheets with 171 rows (up from 163)
- Add new Eng-Sv.xlsx for Swedish
- Add 8 missing strings to all existing spreadsheets (status strings, reflectance, etc.)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -1,32 +1,45 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr codeName="ThisWorkbook"/>
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="Translations" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -41,13 +54,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -194,7 +208,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -229,7 +242,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -264,16 +276,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -395,46 +411,7 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -445,20 +422,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B163"/>
+  <dimension ref="A1:B171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55.83203125" customWidth="1" min="1" max="1"/>
-    <col width="55.83203125" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>German</t>
         </is>
@@ -599,1817 +576,1908 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Weighted</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Gewichtet</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>On</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nein</t>
+          <t>Ein</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Median</t>
+          <t>Off</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Median</t>
+          <t>Aus</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mean</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mittelwert</t>
+          <t>Ja</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>No</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Nein</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Light</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Hell</t>
+          <t>Median</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Dark</t>
+          <t>Mean</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Dunkel</t>
+          <t>Mittelwert</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>File Select</t>
+          <t>System</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dateiauswahl</t>
+          <t>System</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Choose char data file</t>
+          <t>Light</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Datendatei auswählen</t>
+          <t>Hell</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Drop files here</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dateien hier ablegen</t>
+          <t>Dunkel</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>or use button above</t>
+          <t>File Select</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>oder Schaltfläche oben nutzen</t>
+          <t>Dateiauswahl</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sort files alphabetically</t>
+          <t>Choose char data file</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alphabetisch sortieren</t>
+          <t>Datendatei auswählen</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Explore</t>
+          <t>Drop files here</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Erkunden</t>
+          <t>Dateien hier ablegen</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>or use button above</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Vergleichen</t>
+          <t>oder Schaltfläche oben nutzen</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Display File</t>
+          <t>Sort files alphabetically</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Datei anzeigen</t>
+          <t>Alphabetisch sortieren</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Drag files here from</t>
+          <t>Explore</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Dateien hier hinziehen aus</t>
+          <t>Erkunden</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>File Select pane or file system</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dateiauswahl oder Dateisystem</t>
+          <t>Vergleichen</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>3D Plot</t>
+          <t>Display File</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>3D-Diagramm</t>
+          <t>Datei anzeigen</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Controls</t>
+          <t>Drag files here from</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Steuerung</t>
+          <t>Dateien hier hinziehen aus</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Show gamut shell</t>
+          <t>File Select pane or file system</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Gamut-Hülle anzeigen</t>
+          <t>Dateiauswahl oder Dateisystem</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Show data points</t>
+          <t>3D Plot</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Datenpunkte anzeigen</t>
+          <t>3D-Diagramm</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Color by hue angle</t>
+          <t>Controls</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nach Farbton einfärben</t>
+          <t>Steuerung</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Color by value</t>
+          <t>Show gamut shell</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Nach Helligkeit einfärben</t>
+          <t>Gamut-Hülle anzeigen</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Show spectral data when point selected</t>
+          <t>Show data points</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Spektraldaten bei Klick anzeigen</t>
+          <t>Datenpunkte anzeigen</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Computing…</t>
+          <t>Color by hue angle</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Berechnung…</t>
+          <t>Nach Farbton einfärben</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Gamut Slice (2D)</t>
+          <t>Color by value</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Gamut-Schnitt (2D)</t>
+          <t>Nach Helligkeit einfärben</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Axis:</t>
+          <t>Show spectral data when point selected</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Achse:</t>
+          <t>Spektraldaten bei Klick anzeigen</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Value:</t>
+          <t>Computing…</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Wert:</t>
+          <t>Berechnung…</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Bandwidth ±</t>
+          <t>Gamut Slice (2D)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Bandbreite ±</t>
+          <t>Gamut-Schnitt (2D)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>No file loaded</t>
+          <t>Axis:</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Keine Datei geladen</t>
+          <t>Achse:</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tone Value</t>
+          <t>Value:</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Tonwert</t>
+          <t>Wert:</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tone Method</t>
+          <t>No file loaded</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Tonwert-Methode</t>
+          <t>Keine Datei geladen</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Spectral Murray-Davies</t>
+          <t>Tone Value</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Spektral Murray-Davies</t>
+          <t>Tonwert</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Colour Tone Value (CTV)</t>
+          <t>Tone Method</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Farb-Tonwert (CTV)</t>
+          <t>Tonwert-Methode</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Spectral Murray-Davies</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Spektral Murray-Davies</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Graph Type</t>
+          <t>Colour Tone Value (CTV)</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Diagrammtyp</t>
+          <t>Farb-Tonwert (CTV)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Transfer</t>
+          <t>Filter</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Transfer</t>
+          <t>Filter</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Gain</t>
+          <t>Graph Type</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Gewinn</t>
+          <t>Diagrammtyp</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ideal</t>
+          <t>Transfer</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ideal</t>
+          <t>Transfer</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Datasets</t>
+          <t>Gain</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Datensätze</t>
+          <t>Gewinn</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Validate</t>
+          <t>Ideal</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Validieren</t>
+          <t>Ideal</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Comparison Table</t>
+          <t>Datasets</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Vergleichstabelle</t>
+          <t>Datensätze</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Extract</t>
+          <t>Validate</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Extrahieren</t>
+          <t>Validieren</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Restore</t>
+          <t>Comparison Table</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Wiederherstellen</t>
+          <t>Vergleichstabelle</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Export</t>
+          <t>Extract</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Exportieren</t>
+          <t>Extrahieren</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Data Table</t>
+          <t>Restore</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Datentabelle</t>
+          <t>Wiederherstellen</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Schätzung</t>
+          <t>Exportieren</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Primaries</t>
+          <t>Data Table</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Primärfarben</t>
+          <t>Datentabelle</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Secondaries</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Sekundärfarben</t>
+          <t>Schätzung</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CMY Grays</t>
+          <t>Primaries</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CMY-Grautöne</t>
+          <t>Primärfarben</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CMY Browns</t>
+          <t>Secondaries</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CMY-Brauntöne</t>
+          <t>Sekundärfarben</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Solids Only</t>
+          <t>CMY Grays</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Nur Vollfarben</t>
+          <t>CMY-Grautöne</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Remove paper white point</t>
+          <t>CMY Browns</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Papierweißpunkt entfernen</t>
+          <t>CMY-Brauntöne</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Remove selected colorants from data.</t>
+          <t>Solids Only</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Ausgewählte Farbmittel aus den Daten entfernen.</t>
+          <t>Nur Vollfarben</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Export File</t>
+          <t>Remove paper white point</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Datei exportieren</t>
+          <t>Papierweißpunkt entfernen</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Folder</t>
+          <t>Remove selected colorants from data.</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Ordner</t>
+          <t>Ausgewählte Farbmittel aus den Daten entfernen.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>File name</t>
+          <t>Export File</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Dateiname</t>
+          <t>Datei exportieren</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Format</t>
+          <t>Folder</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Format</t>
+          <t>Ordner</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>File name</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Abbrechen</t>
+          <t>Dateiname</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Save</t>
+          <t>Format</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Speichern</t>
+          <t>Format</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Select folder</t>
+          <t>Cancel</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Ordner auswählen</t>
+          <t>Abbrechen</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Browse for folder</t>
+          <t>Save</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ordner durchsuchen</t>
+          <t>Speichern</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Folder picker not supported in this browser</t>
+          <t>Select folder</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Ordnerauswahl wird von diesem Browser nicht unterstützt</t>
+          <t>Ordner auswählen</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Export destination folder…</t>
+          <t>Browse for folder</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Zielordner…</t>
+          <t>Ordner durchsuchen</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>File is neither CSV nor CGATS/ISO28178 format</t>
+          <t>Folder picker not supported in this browser</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Datei ist weder CSV noch CGATS/ISO28178</t>
+          <t>Ordnerauswahl wird von diesem Browser nicht unterstützt</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>✓ Valid</t>
+          <t>File Select: Drop or load files here to select.</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>✓ Gültig</t>
+          <t>Dateiauswahl: Dateien hier ablegen oder laden.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>LAB computed from spectral ({ill} / {obs} / {mc})</t>
+          <t>Drag-and-drop files from file system or File Select here</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>LAB aus Spektraldaten ({ill} / {obs} / {mc})</t>
+          <t>Dateien vom Dateisystem oder der Dateiauswahl hierher ziehen</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Missing: {cols}</t>
+          <t>Click to sort</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Fehlend: {cols}</t>
+          <t>Zum Sortieren klicken</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Loaded {n} rows.</t>
+          <t>Click to view spectral</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>{n} Zeilen geladen.</t>
+          <t>Klicken für Spektrum</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Loaded {n} rows, reduced to {m} rows by filtering duplicates ({method}).</t>
+          <t>Toggle controls</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>{n} Zeilen geladen, auf {m} durch Duplikatfilter ({method}) reduziert.</t>
+          <t>Steuerung ein-/ausblenden</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Device colorants:</t>
+          <t>Remove {item}</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Gerätefarbmittel:</t>
+          <t>{item} entfernen</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Device colorants: none</t>
+          <t>Click to toggle on/off</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Gerätefarbmittel: keine</t>
+          <t>Klicken zum Ein-/Ausschalten</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>File contains spectral data. Click on data points to display spectral graph.</t>
+          <t>Export destination folder…</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Datei enthält Spektraldaten. Auf Datenpunkte klicken für Spektraldiagramm.</t>
+          <t>Zielordner…</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Colorimetric only. No spectral data found in file.</t>
+          <t>File is neither CSV nor CGATS/ISO28178 format</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Nur colorimetrisch. Keine Spektraldaten in der Datei gefunden.</t>
+          <t>Datei ist weder CSV noch CGATS/ISO28178</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>{n} rows (after extract).</t>
+          <t>File header is not standard CGATS (first line does not contain “CGATS” or “ISO28178”)</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>{n} Zeilen (nach Extraktion).</t>
+          <t>Dateikopfzeile entspricht nicht Standard-CGATS (erste Zeile enthält weder „CGATS“ noch „ISO28178“)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>No comparable inkings between selected files.</t>
+          <t>✓ Valid</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Keine vergleichbaren Farbanteile in den ausgewählten Dateien.</t>
+          <t>✓ Gültig</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>{n} matching data point</t>
+          <t>LAB computed from spectral ({ill} / {obs} / {mc})</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>{n} übereinstimmender Datenpunkt</t>
+          <t>LAB aus Spektraldaten ({ill} / {obs} / {mc})</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>{n} matching data points</t>
+          <t>Missing: {cols}</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>{n} übereinstimmende Datenpunkte</t>
+          <t>Fehlend: {cols}</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Mean {method}</t>
+          <t>Loaded {n} rows.</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Mittel {method}</t>
+          <t>{n} Zeilen geladen.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Min {method}</t>
+          <t>Loaded {n} rows, reduced to {m} rows by filtering duplicates ({method}).</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Min {method}</t>
+          <t>{n} Zeilen geladen, auf {m} durch Duplikatfilter ({method}) reduziert.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Max {method}</t>
+          <t>Device colorants:</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Max {method}</t>
+          <t>Gerätefarbmittel:</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Std Dev</t>
+          <t>Device colorants: none</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Std.-Abw.</t>
+          <t>Gerätefarbmittel: keine</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Device Colorants</t>
+          <t>File contains spectral data. Click on data points to display spectral graph.</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Gerätefarbmittel</t>
+          <t>Datei enthält Spektraldaten. Auf Datenpunkte klicken für Spektraldiagramm.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Difference</t>
+          <t>Colorimetric only. No spectral data found in file.</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Differenz</t>
+          <t>Nur colorimetrisch. Keine Spektraldaten in der Datei gefunden.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Opacity</t>
+          <t>{n} rows (after extract).</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Deckkraft</t>
+          <t>{n} Zeilen (nach Extraktion).</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>↻ Regenerate Shell</t>
+          <t>No comparable inkings between selected files.</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>↻ Hülle neu erstellen</t>
+          <t>Keine vergleichbaren Farbanteile in den ausgewählten Dateien.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Mesh</t>
+          <t>{n} matching data point</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Netz</t>
+          <t>{n} übereinstimmender Datenpunkt</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Density</t>
+          <t>{n} matching data points</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Dichte</t>
+          <t>{n} übereinstimmende Datenpunkte</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Lighting</t>
+          <t>Mean {method}</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Beleuchtung</t>
+          <t>Mittel {method}</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ambient</t>
+          <t>Min {method}</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Umgebung</t>
+          <t>Min {method}</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>diffuse</t>
+          <t>Max {method}</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>diffus</t>
+          <t>Max {method}</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>specular</t>
+          <t>Std Dev</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>spekular</t>
+          <t>Std.-Abw.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>roughness</t>
+          <t>Points fitted</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Rauheit</t>
+          <t>Angepasste Punkte</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Dataset Settings</t>
+          <t>Dataset {slot}</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Datensatzeinstellungen</t>
+          <t>Datensatz {slot}</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Select to toggle file visibility:</t>
+          <t>Device Colorants</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Klicken zum Ein-/Ausblenden:</t>
+          <t>Gerätefarbmittel</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Toggle:</t>
+          <t>Difference</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Anzeigen:</t>
+          <t>Differenz</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Show:</t>
+          <t>Opacity</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Ansicht:</t>
+          <t>Deckkraft</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>↻ Regenerate Shell</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Original</t>
+          <t>↻ Hülle neu erstellen</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Modified</t>
+          <t>Mesh</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Geändert</t>
+          <t>Netz</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>✕ Close</t>
+          <t>Density</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>✕ Schließen</t>
+          <t>Dichte</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Selected file is not loaded.</t>
+          <t>Lighting</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Ausgewählte Datei ist nicht geladen.</t>
+          <t>Beleuchtung</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Both files must be loaded.</t>
+          <t>ambient</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Beide Dateien müssen geladen sein.</t>
+          <t>Umgebung</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>No K-only patches matched.</t>
+          <t>diffuse</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Keine K-Einzel-Patches gefunden.</t>
+          <t>diffus</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>No CMY patches matched.</t>
+          <t>specular</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Keine CMY-Patches gefunden.</t>
+          <t>spekular</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Missing CMYK device colorants in Dataset A{name}.</t>
+          <t>roughness</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Fehlende CMYK-Farbmittel in Datensatz A{name}.</t>
+          <t>Rauheit</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Missing L*a*b* data in Dataset A{name}.</t>
+          <t>Dataset Settings</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Fehlende L*a*b*-Daten in Datensatz A{name}.</t>
+          <t>Datensatzeinstellungen</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Paper white patch (0,0,0,0) not found in Dataset A.</t>
+          <t>Select to toggle file visibility:</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Papierweißpatch (0,0,0,0) nicht in Datensatz A gefunden.</t>
+          <t>Klicken zum Ein-/Ausblenden:</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>100K solid patch not found in Dataset A.</t>
+          <t>Toggle:</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>100K-Vollpatch nicht in Datensatz A gefunden.</t>
+          <t>Anzeigen:</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>100CMY solid patch not found in Dataset A.</t>
+          <t>Show:</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>100CMY-Vollpatch nicht in Datensatz A gefunden.</t>
+          <t>Ansicht:</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>G7 Overall:</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>G7 Gesamt:</t>
+          <t>Original</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Scale</t>
+          <t>Modified</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Skala</t>
+          <t>Geändert</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Tolerance</t>
+          <t>✕ Close</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Toleranz</t>
+          <t>✕ Schließen</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>K (Black)</t>
+          <t>Selected file is not loaded.</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>K (Schwarz)</t>
+          <t>Ausgewählte Datei ist nicht geladen.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>K patches ({n})</t>
+          <t>Both files must be loaded.</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>K-Patches ({n})</t>
+          <t>Beide Dateien müssen geladen sein.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>CMY patches ({n})</t>
+          <t>No K-only patches matched.</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>CMY-Patches ({n})</t>
+          <t>Keine K-Einzel-Patches gefunden.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>K%</t>
+          <t>No CMY patches matched.</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>K %</t>
+          <t>Keine CMY-Patches gefunden.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>L* meas</t>
+          <t>Missing CMYK device colorants in Dataset A{name}.</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>L* gemessen</t>
+          <t>Fehlende CMYK-Farbmittel in Datensatz A{name}.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>L* aim</t>
+          <t>Missing L*a*b* data in Dataset A{name}.</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>L* Zielwert</t>
+          <t>Fehlende L*a*b*-Daten in Datensatz A{name}.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>meas</t>
+          <t>Paper white patch (0,0,0,0) not found in Dataset A.</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>gem.</t>
+          <t>Papierweißpatch (0,0,0,0) nicht in Datensatz A gefunden.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>aim</t>
+          <t>100K solid patch not found in Dataset A.</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Ziel</t>
+          <t>100K-Vollpatch nicht in Datensatz A gefunden.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>No spectral data — switch to Colour Tone Value (CTV)</t>
+          <t>100CMY solid patch not found in Dataset A.</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Keine Spektraldaten — auf Farb-Tonwert (CTV) wechseln</t>
+          <t>100CMY-Vollpatch nicht in Datensatz A gefunden.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>No primary tone steps found.
-Needs rows with a single non-zero colorant.</t>
+          <t>G7 Overall:</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Keine Primär-Tonstufen gefunden.
-Es werden Zeilen mit einem einzigen Farbmittel benötigt.</t>
+          <t>G7 Gesamt:</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Tone Value Gain (%)</t>
+          <t>Scale</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Tonwertzuwachs (%)</t>
+          <t>Skala</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Tone Value (%)</t>
+          <t>Tolerance</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Tonwert (%)</t>
+          <t>Toleranz</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Input (%)</t>
+          <t>K (Black)</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Eingabe (%)</t>
+          <t>K (Schwarz)</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Model fit — degree {deg}, {n} points</t>
+          <t>K patches ({n})</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Modellanpassung — Grad {deg}, {n} Punkte</t>
+          <t>K-Patches ({n})</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>↻ Regenerate</t>
+          <t>CMY patches ({n})</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>↻ Neu erstellen</t>
+          <t>CMY-Patches ({n})</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Input colorant</t>
+          <t>K%</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Eingabe
-Farbmittel</t>
+          <t>K %</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Nearest
-in dataset</t>
+          <t>L* meas</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Nächster
-im Datensatz</t>
+          <t>L* gemessen</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>L* aim</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Modell</t>
+          <t>L* Zielwert</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Computing…</t>
+          <t>meas</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Berechnung…</t>
+          <t>gem.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Model fit failed: {msg}</t>
+          <t>aim</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Modellanpassung fehlgeschlagen: {msg}</t>
+          <t>Ziel</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Retry</t>
+          <t>No spectral data — switch to Colour Tone Value (CTV)</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Wiederholen</t>
+          <t>Keine Spektraldaten — auf Farb-Tonwert (CTV) wechseln</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Click on L*a*b* color to display spectral graph.</t>
+          <t>No primary tone steps found.\nNeeds rows with a single non-zero colorant.</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Auf L*a*b*-Farbe klicken für Spektraldiagramm.</t>
+          <t>Keine Primär-Tonstufen gefunden.\nEs werden Zeilen mit einem einzigen Farbmittel benötigt.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Scroll to top</t>
+          <t>Tone Value Gain (%)</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Nach oben</t>
+          <t>Tonwertzuwachs (%)</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Help</t>
+          <t>Tone Value (%)</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Hilfe</t>
+          <t>Tonwert (%)</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>About CharData</t>
+          <t>Input (%)</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Über CharData</t>
+          <t>Eingabe (%)</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Support on Ko-fi</t>
+          <t>Model fit — degree {deg}, {n} points</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Ko-fi unterstützen</t>
+          <t>Modellanpassung — Grad {deg}, {n} Punkte</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CharData is free for the color community. If it helps you, a small Ko-fi donation helps keep it running.</t>
+          <t>↻ Regenerate</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>CharData ist für die Farbgemeinschaft kostenlos. Eine kleine Ko-fi-Spende hilft, den Dienst am Laufen zu halten.</t>
+          <t>↻ Neu erstellen</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Points fitted</t>
+          <t>Input\ncolorant</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Angepasste Punkte</t>
+          <t>Eingabe\nFarbmittel</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Dataset {slot}</t>
+          <t>Nearest\nin dataset</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Datensatz {slot}</t>
+          <t>Nächster\nim Datensatz</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>File Select: Drop or load files here to select.</t>
+          <t>Model</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Dateiauswahl: Dateien hier ablegen oder laden.</t>
+          <t>Modell</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Drag-and-drop files from file system or File Select here</t>
+          <t>Computing…</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Dateien vom Dateisystem oder der Dateiauswahl hierher ziehen</t>
+          <t>Berechnung…</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Click to sort</t>
+          <t>Calculating tone values…</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Zum Sortieren klicken</t>
+          <t>Calculating tone values…</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Click to view spectral</t>
+          <t>Estimating model…</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Klicken für Spektrum</t>
+          <t>Estimating model…</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Toggle controls</t>
+          <t>Building 3D gamut…</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Steuerung ein-/ausblenden</t>
+          <t>Building 3D gamut…</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Remove {item}</t>
+          <t>Computing 2D slice…</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>{item} entfernen</t>
+          <t>Computing 2D slice…</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Click to toggle on/off</t>
+          <t>Rendering…</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Klicken zum Ein-/Ausschalten</t>
+          <t>Rendering…</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Model fit failed: {msg}</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Oben</t>
+          <t>Modellanpassung fehlgeschlagen: {msg}</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Buy me a coffee</t>
+          <t>Retry</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Kauf mir einen Kaffee</t>
+          <t>Wiederholen</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>File header is not standard CGATS (first line does not contain “CGATS” or “ISO28178”)</t>
+          <t>Click on L*a*b* color to display spectral graph.</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Dateikopfzeile entspricht nicht Standard-CGATS (erste Zeile enthält weder „CGATS“ noch „ISO28178“)</t>
+          <t>Auf L*a*b*-Farbe klicken für Spektraldiagramm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Scroll to top</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Nach oben</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Oben</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Help</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Hilfe</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>About CharData</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Über CharData</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Support on Ko-fi</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Ko-fi unterstützen</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Buy me a coffee</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Kauf mir einen Kaffee</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Reflectance</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Reflexionsgrad</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>CharData is free for the color community. If it helps you, a small Ko-fi donation helps keep it running.</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>CharData ist für die Farbgemeinschaft kostenlos. Eine kleine Ko-fi-Spende hilft, den Dienst am Laufen zu halten.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Translate Standard Datasets strings; document in MANUAL.md
- MANUAL.md "Loading datasets": describe the new Standard datasets
  collapsible section (defaults collapsed; clicks load through the
  same pipeline as user files).
- I18N dict: add fs_section_std, fs_loading_std, fs_load_std_failed
  to all 11 non-EN languages (fr, de, it, es, pt-PT, pt-BR, zh-CN,
  zh-TW, ja, ko, sv).
- translations/Eng-*.xlsx: append matching rows to the 9 canonical
  spreadsheets so the audit and the dict stay in sync.
- public/help.html regenerated from MANUAL.md by the pre-commit hook.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B178"/>
+  <dimension ref="A1:B181"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1825,9 +1825,33 @@
         <v>Kein gültiges ICC-Profil (Header-Signatur fehlt).</v>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>Standard datasets</v>
+      </c>
+      <c r="B179" t="str">
+        <v>Standarddatensätze</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>Loading…</v>
+      </c>
+      <c r="B180" t="str">
+        <v>Wird geladen…</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>Failed to load list</v>
+      </c>
+      <c r="B181" t="str">
+        <v>Liste konnte nicht geladen werden</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B178"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B181"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Drag-and-drop standard datasets; restyle File Select label
Standard dataset rows are now draggable: a dragstart handler sets a
'std-dataset-fname' payload, and the panel drop handler fetches the
file and routes it through addFileToList.

File Select pane: removed the standalone "File Select" header and
folded the title into the load button (15px bold, left-aligned),
with the file kinds reflowed onto separate lines below. choose_file
i18n + the 9 Eng-*.xlsx spreadsheets updated to match.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -585,12 +585,12 @@
     </row>
     <row r="24" xml:space="preserve">
       <c r="A24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Select files:
-characterization data or ICC profiles</v>
+        <v xml:space="preserve">characterization data
+or ICC profiles</v>
       </c>
       <c r="B24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Dateien auswählen:
-Charakterisierungsdaten oder ICC-Profile</v>
+        <v xml:space="preserve">Charakterisierungsdaten
+oder ICC-Profile</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Translate slicer controls; document Thickness/Fall-off/points
Adds Thickness, Fall-off (Hard/Soft), Hard, Soft strings to the I18N
dict for fr, de, it, es, pt-PT, pt-BR, zh-CN, zh-TW, ja, ko, sv. The
9 active Eng-*.xlsx spreadsheets get the same four new rows. The new
show_data_points key reuses the existing "Show data points" string,
so no spreadsheet row is needed.

MANUAL.md: replaced the unimplemented "Bandwidth ±" entry with the
real Thickness, Fall-off, and Show data points rows, describing the
±0.5 full-opacity window and the marker-size split. help.html is
regenerated from this by the pre-commit hook.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B181"/>
+  <dimension ref="A1:B185"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1849,9 +1849,41 @@
         <v>Liste konnte nicht geladen werden</v>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>Thickness:</v>
+      </c>
+      <c r="B182" t="str">
+        <v>Dicke:</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>Fall-off:</v>
+      </c>
+      <c r="B183" t="str">
+        <v>Übergang:</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>Hard</v>
+      </c>
+      <c r="B184" t="str">
+        <v>Hart</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>Soft</v>
+      </c>
+      <c r="B185" t="str">
+        <v>Weich</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B181"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B185"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Re-translate dataset type label and compare/G7 error strings on lang change
refreshPanelUI now re-localizes the type label for CSV/CGATS data
(previously only the ICC path was handled), so "Characterization
dataset" updates when the language changes. The CSV vs CGATS choice
is now persisted on state[slot].isCSV.

onLangChange triggers renderSlicePlot() so the slice tab label suffix
("— L* = 50") and legend tooltip pick up the new language without
needing a slider nudge.

Four hardcoded English error strings replaced with t() calls and
new i18n keys (g7_not_for_icc, icc_vs_icc_cmyk_only, cmp_b_no_match_a,
cmp_a_no_match_b), translated for fr/de/it/es/pt-PT/pt-BR/zh-CN/zh-TW/
ja/ko/sv. Eng-*.xlsx spreadsheets get the matching rows.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B185"/>
+  <dimension ref="A1:B189"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1881,9 +1881,41 @@
         <v>Weich</v>
       </c>
     </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>G7 validation is not available for ICC profiles.</v>
+      </c>
+      <c r="B186" t="str">
+        <v>G7-Validierung ist für ICC-Profile nicht verfügbar.</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>ICC vs ICC comparison requires CMYK profiles.</v>
+      </c>
+      <c r="B187" t="str">
+        <v>ICC-zu-ICC-Vergleich erfordert CMYK-Profile.</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>Dataset B does not contain colorants matching ICC profile A.</v>
+      </c>
+      <c r="B188" t="str">
+        <v>Datensatz B enthält keine Farbmittel, die zum ICC-Profil A passen.</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>Dataset A does not contain colorants matching ICC profile B.</v>
+      </c>
+      <c r="B189" t="str">
+        <v>Datensatz A enthält keine Farbmittel, die zum ICC-Profil B passen.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B185"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B189"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Launch editor button: hand ICC profile off to icctools via postMessage
- New 'Launch editor' button in the ICC viewer overlay opens icctools in
  a new tab (localhost:5173 in dev, /profiletool/ in prod) and posts the
  profile bytes after the icctools:ready handshake. One-way — icctools
  owns the editing session from there.
- Relax helmet's COOP from 'same-origin' to 'same-origin-allow-popups' so
  cross-origin popups in local dev retain window.opener. Prod is same-origin
  (/profiletool/ subpath) so this is a no-op there.
- i18n + 9 translation xlsx files updated with icc_launch_editor.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B192"/>
+  <dimension ref="A1:B193"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1937,9 +1937,17 @@
         <v>ICC-Viewer wird geladen…</v>
       </c>
     </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>Launch editor</v>
+      </c>
+      <c r="B193" t="str">
+        <v>Editor öffnen</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B192"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B193"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add page title + "data stays local" hint with translations
- New page heading "Chardata Viewer" with subtitle "Free browser-resident
  online tool" above the Explore/Compare segment row.
- New right-aligned, light-yellow note "All data stays local to browser"
  under the existing drop hint in each panel's empty state, with
  vertical spacing so it doesn't blur into the drop hint.
- Translated app_subtitle and local_only_note across all 11 non-EN
  locales; appended matching rows to each translations/Eng-*.xlsx
  (preserving existing translator content).
- MANUAL.md intro now explicitly notes "no upload to any server"; help.html
  regenerated by the pre-commit hook.
- Dark-mode tweaks for the new title (#e0e0e0) and the yellow note
  (#d4b85a) so they read against the dark background.
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B193"/>
+  <dimension ref="A1:B195"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1945,9 +1945,25 @@
         <v>Editor öffnen</v>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>All data stays local to browser</v>
+      </c>
+      <c r="B194" t="str">
+        <v>Alle Daten bleiben lokal im Browser</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>Free browser-resident online tool</v>
+      </c>
+      <c r="B195" t="str">
+        <v>Kostenloses Online-Tool, das im Browser läuft</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B193"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B195"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix translation drift: literal \n → real newlines in xlsx
Three I18N keys (no_primary_steps, colorant_input, nearest_dataset) use
embedded newlines for line breaks in UI labels and error messages. The
xlsx files had stored those as the two-character escape sequence "\n"
instead of an actual newline, so check-translations.js flagged the EN
column as drift on every locale.

Replaced literal "\n" with real newlines across all cells in all 9
spreadsheets. Audit now reports zero drift.
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -1561,12 +1561,14 @@
         <v>Keine Spektraldaten — auf Farb-Tonwert (CTV) wechseln</v>
       </c>
     </row>
-    <row r="146">
-      <c r="A146" t="str">
-        <v>No primary tone steps found.\nNeeds rows with a single non-zero colorant.</v>
-      </c>
-      <c r="B146" t="str">
-        <v>Keine Primär-Tonstufen gefunden.\nEs werden Zeilen mit einem einzigen Farbmittel benötigt.</v>
+    <row r="146" xml:space="preserve">
+      <c r="A146" t="str" xml:space="preserve">
+        <v xml:space="preserve">No primary tone steps found.
+Needs rows with a single non-zero colorant.</v>
+      </c>
+      <c r="B146" t="str" xml:space="preserve">
+        <v xml:space="preserve">Keine Primär-Tonstufen gefunden.
+Es werden Zeilen mit einem einzigen Farbmittel benötigt.</v>
       </c>
     </row>
     <row r="147">
@@ -1609,20 +1611,24 @@
         <v>↻ Neu erstellen</v>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" t="str">
-        <v>Input\ncolorant</v>
-      </c>
-      <c r="B152" t="str">
-        <v>Eingabe\nFarbmittel</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="str">
-        <v>Nearest\nin dataset</v>
-      </c>
-      <c r="B153" t="str">
-        <v>Nächster\nim Datensatz</v>
+    <row r="152" xml:space="preserve">
+      <c r="A152" t="str" xml:space="preserve">
+        <v xml:space="preserve">Input
+colorant</v>
+      </c>
+      <c r="B152" t="str" xml:space="preserve">
+        <v xml:space="preserve">Eingabe
+Farbmittel</v>
+      </c>
+    </row>
+    <row r="153" xml:space="preserve">
+      <c r="A153" t="str" xml:space="preserve">
+        <v xml:space="preserve">Nearest
+in dataset</v>
+      </c>
+      <c r="B153" t="str" xml:space="preserve">
+        <v xml:space="preserve">Nächster
+im Datensatz</v>
       </c>
     </row>
     <row r="154">

</xml_diff>

<commit_message>
1.7.0: Image gamut feature
Compare-mode workflow to load a PNG/JPEG/TIFF image, derive its
device-space colorimetry, and plot its gamut as a green point cloud
overlaid on the existing Dataset A / Dataset B traces in the 3D plot
and 2D slice. For non-Lab images, the user binds to A or B; the
dataset's estimate model (char data) or A2B with Absolute Colorimetric
intent (ICC) converts device pixels to L*a*b*. Lab TIFFs plot directly.

JPEG/TIFF embedded ICC profiles are read for color-space detection;
PNG falls back to channel-count inference. UTIF.js is vendored under
public/lib/ for TIFF decode incl. CIELAB photometric.

server.js: allow blob: in CSP img-src so URL.createObjectURL() works
in the <img> decode path.

i18n: ten new image_* keys added to all 12 locale dicts and the nine
active translation spreadsheets; translations audit clean.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B195"/>
+  <dimension ref="A1:B205"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1967,9 +1967,89 @@
         <v>Kostenloses Online-Tool, das im Browser läuft</v>
       </c>
     </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>Image</v>
+      </c>
+      <c r="B196" t="str">
+        <v>Bild</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>Load Image</v>
+      </c>
+      <c r="B197" t="str">
+        <v>Bild laden</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>Bind image to dataset</v>
+      </c>
+      <c r="B198" t="str">
+        <v>Bild mit Datensatz verknüpfen</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>Remove image</v>
+      </c>
+      <c r="B199" t="str">
+        <v>Bild entfernen</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>Image color space: {cs} {src}</v>
+      </c>
+      <c r="B200" t="str">
+        <v>Bildfarbraum: {cs} {src}</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>Bound to {name} — {n} points</v>
+      </c>
+      <c r="B201" t="str">
+        <v>Verknüpft mit {name} — {n} Punkte</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>Lab image — {n} points</v>
+      </c>
+      <c r="B202" t="str">
+        <v>Lab-Bild — {n} Punkte</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>Cannot bind: image is {img} but Dataset {slot} is {family}.</v>
+      </c>
+      <c r="B203" t="str">
+        <v>Verknüpfung nicht möglich: Bild ist {img}, aber Datensatz {slot} ist {family}.</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>Unsupported image format. Use PNG, JPEG, or TIFF.</v>
+      </c>
+      <c r="B204" t="str">
+        <v>Bildformat nicht unterstützt. Bitte PNG, JPEG oder TIFF verwenden.</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>“{name}” is too large ({mb} MB). Maximum image size is {max} MB.</v>
+      </c>
+      <c r="B205" t="str">
+        <v>„{name}“ ist zu groß ({mb} MB). Maximale Bildgröße: {max} MB.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B195"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B205"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Subscribe consent: link to colourbill privacy notice
Restructures the consent label inside the subscribe modal to include a
"Privacy notice" link pointing at https://www.colourbill.com/privacy/.
The link text is itself translated (new sub_privacy_link i18n key) in
all 12 languages, with matching rows appended to every live
translations/Eng-*.xlsx.

Touchpoints:
- public/index.html: modal markup now nests a sub_privacy_link <a> next
  to the sub_consent span (separate elements so applyTranslations'
  textContent doesn't strip the anchor).
- I18N dict: sub_privacy_link added in en/fr/de/it/es/pt-PT/pt-BR/
  zh-CN/zh-TW/ja/ko/sv.
- translations/Eng-*.xlsx: matching rows. check-translations.js reports
  zero drift across all live spreadsheets.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B263"/>
+  <dimension ref="A1:B264"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2511,9 +2511,17 @@
         <v>Schließen</v>
       </c>
     </row>
+    <row r="264">
+      <c r="A264" t="str">
+        <v>Privacy notice</v>
+      </c>
+      <c r="B264" t="str">
+        <v>Datenschutzhinweis</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B263"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B264"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove redundant "Regenerate Shell" button from gamut panel
The button rebuilt the shell at the fixed default BOUNDARY_STEPS, ignoring
the Density slider, and produced an identical mesh from the (deterministic)
loaded data — every input change (file load, rendering intent, model weights,
density) already triggers its own rebuild path, so the button was vestigial.
The Density slider is now the sole interactive resolution control.

regenerateGamutShell() stays (still called internally by setRenderingIntent).
Drops the now-orphan regen_shell string from all 12 I18N dicts and the 9
translation spreadsheets. check-translations.js reports 0 drift.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B269"/>
+  <dimension ref="A1:B268"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1275,1293 +1275,1285 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>↻ Regenerate Shell</v>
+        <v>Mesh</v>
       </c>
       <c r="B110" t="str">
-        <v>↻ Hülle neu erstellen</v>
+        <v>Netz</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Mesh</v>
+        <v>Density</v>
       </c>
       <c r="B111" t="str">
-        <v>Netz</v>
+        <v>Dichte</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>Density</v>
+        <v>Lighting</v>
       </c>
       <c r="B112" t="str">
-        <v>Dichte</v>
+        <v>Beleuchtung</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>Lighting</v>
+        <v>ambient</v>
       </c>
       <c r="B113" t="str">
-        <v>Beleuchtung</v>
+        <v>Umgebung</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>ambient</v>
+        <v>diffuse</v>
       </c>
       <c r="B114" t="str">
-        <v>Umgebung</v>
+        <v>diffus</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>diffuse</v>
+        <v>specular</v>
       </c>
       <c r="B115" t="str">
-        <v>diffus</v>
+        <v>spekular</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>specular</v>
+        <v>roughness</v>
       </c>
       <c r="B116" t="str">
-        <v>spekular</v>
+        <v>Rauheit</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>roughness</v>
+        <v>Dataset Settings</v>
       </c>
       <c r="B117" t="str">
-        <v>Rauheit</v>
+        <v>Datensatzeinstellungen</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Dataset Settings</v>
+        <v>Select to toggle file visibility:</v>
       </c>
       <c r="B118" t="str">
-        <v>Datensatzeinstellungen</v>
+        <v>Klicken zum Ein-/Ausblenden:</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Select to toggle file visibility:</v>
+        <v>Toggle:</v>
       </c>
       <c r="B119" t="str">
-        <v>Klicken zum Ein-/Ausblenden:</v>
+        <v>Anzeigen:</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>Toggle:</v>
+        <v>Show:</v>
       </c>
       <c r="B120" t="str">
-        <v>Anzeigen:</v>
+        <v>Ansicht:</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>Show:</v>
+        <v>Original</v>
       </c>
       <c r="B121" t="str">
-        <v>Ansicht:</v>
+        <v>Original</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>Original</v>
+        <v>Modified</v>
       </c>
       <c r="B122" t="str">
-        <v>Original</v>
+        <v>Geändert</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>Modified</v>
+        <v>✕ Close</v>
       </c>
       <c r="B123" t="str">
-        <v>Geändert</v>
+        <v>✕ Schließen</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>✕ Close</v>
+        <v>Selected file is not loaded.</v>
       </c>
       <c r="B124" t="str">
-        <v>✕ Schließen</v>
+        <v>Ausgewählte Datei ist nicht geladen.</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>Selected file is not loaded.</v>
+        <v>Both files must be loaded.</v>
       </c>
       <c r="B125" t="str">
-        <v>Ausgewählte Datei ist nicht geladen.</v>
+        <v>Beide Dateien müssen geladen sein.</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>Both files must be loaded.</v>
+        <v>No K-only patches matched.</v>
       </c>
       <c r="B126" t="str">
-        <v>Beide Dateien müssen geladen sein.</v>
+        <v>Keine K-Einzel-Patches gefunden.</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>No K-only patches matched.</v>
+        <v>No CMY patches matched.</v>
       </c>
       <c r="B127" t="str">
-        <v>Keine K-Einzel-Patches gefunden.</v>
+        <v>Keine CMY-Patches gefunden.</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>No CMY patches matched.</v>
+        <v>Missing CMYK device colorants in Dataset A{name}.</v>
       </c>
       <c r="B128" t="str">
-        <v>Keine CMY-Patches gefunden.</v>
+        <v>Fehlende CMYK-Farbmittel in Datensatz A{name}.</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>Missing CMYK device colorants in Dataset A{name}.</v>
+        <v>Missing L*a*b* data in Dataset A{name}.</v>
       </c>
       <c r="B129" t="str">
-        <v>Fehlende CMYK-Farbmittel in Datensatz A{name}.</v>
+        <v>Fehlende L*a*b*-Daten in Datensatz A{name}.</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>Missing L*a*b* data in Dataset A{name}.</v>
+        <v>Paper white patch (0,0,0,0) not found in Dataset A.</v>
       </c>
       <c r="B130" t="str">
-        <v>Fehlende L*a*b*-Daten in Datensatz A{name}.</v>
+        <v>Papierweißpatch (0,0,0,0) nicht in Datensatz A gefunden.</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>Paper white patch (0,0,0,0) not found in Dataset A.</v>
+        <v>100K solid patch not found in Dataset A.</v>
       </c>
       <c r="B131" t="str">
-        <v>Papierweißpatch (0,0,0,0) nicht in Datensatz A gefunden.</v>
+        <v>100K-Vollpatch nicht in Datensatz A gefunden.</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>100K solid patch not found in Dataset A.</v>
+        <v>100CMY solid patch not found in Dataset A.</v>
       </c>
       <c r="B132" t="str">
-        <v>100K-Vollpatch nicht in Datensatz A gefunden.</v>
+        <v>100CMY-Vollpatch nicht in Datensatz A gefunden.</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>100CMY solid patch not found in Dataset A.</v>
+        <v>G7 Overall:</v>
       </c>
       <c r="B133" t="str">
-        <v>100CMY-Vollpatch nicht in Datensatz A gefunden.</v>
+        <v>G7 Gesamt:</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>G7 Overall:</v>
+        <v>Scale</v>
       </c>
       <c r="B134" t="str">
-        <v>G7 Gesamt:</v>
+        <v>Skala</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Scale</v>
+        <v>Tolerance</v>
       </c>
       <c r="B135" t="str">
-        <v>Skala</v>
+        <v>Toleranz</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>Tolerance</v>
+        <v>K (Black)</v>
       </c>
       <c r="B136" t="str">
-        <v>Toleranz</v>
+        <v>K (Schwarz)</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>K (Black)</v>
+        <v>K patches ({n})</v>
       </c>
       <c r="B137" t="str">
-        <v>K (Schwarz)</v>
+        <v>K-Patches ({n})</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>K patches ({n})</v>
+        <v>CMY patches ({n})</v>
       </c>
       <c r="B138" t="str">
-        <v>K-Patches ({n})</v>
+        <v>CMY-Patches ({n})</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>CMY patches ({n})</v>
+        <v>K%</v>
       </c>
       <c r="B139" t="str">
-        <v>CMY-Patches ({n})</v>
+        <v>K %</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>K%</v>
+        <v>L* meas</v>
       </c>
       <c r="B140" t="str">
-        <v>K %</v>
+        <v>L* gemessen</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>L* meas</v>
+        <v>L* aim</v>
       </c>
       <c r="B141" t="str">
-        <v>L* gemessen</v>
+        <v>L* Zielwert</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>L* aim</v>
+        <v>meas</v>
       </c>
       <c r="B142" t="str">
-        <v>L* Zielwert</v>
+        <v>gem.</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>meas</v>
+        <v>aim</v>
       </c>
       <c r="B143" t="str">
-        <v>gem.</v>
+        <v>Ziel</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>aim</v>
+        <v>No spectral data — switch to Colour Tone Value (CTV)</v>
       </c>
       <c r="B144" t="str">
-        <v>Ziel</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="str">
-        <v>No spectral data — switch to Colour Tone Value (CTV)</v>
-      </c>
-      <c r="B145" t="str">
         <v>Keine Spektraldaten — auf Farb-Tonwert (CTV) wechseln</v>
       </c>
     </row>
-    <row r="146" xml:space="preserve">
-      <c r="A146" t="str" xml:space="preserve">
+    <row r="145" xml:space="preserve">
+      <c r="A145" t="str" xml:space="preserve">
         <v xml:space="preserve">No primary tone steps found.
 Needs rows with a single non-zero colorant.</v>
       </c>
-      <c r="B146" t="str" xml:space="preserve">
+      <c r="B145" t="str" xml:space="preserve">
         <v xml:space="preserve">Keine Primär-Tonstufen gefunden.
 Es werden Zeilen mit einem einzigen Farbmittel benötigt.</v>
       </c>
     </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>Tone Value Gain (%)</v>
+      </c>
+      <c r="B146" t="str">
+        <v>Tonwertzuwachs (%)</v>
+      </c>
+    </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>Tone Value Gain (%)</v>
+        <v>Tone Value (%)</v>
       </c>
       <c r="B147" t="str">
-        <v>Tonwertzuwachs (%)</v>
+        <v>Tonwert (%)</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>Tone Value (%)</v>
+        <v>Input (%)</v>
       </c>
       <c r="B148" t="str">
-        <v>Tonwert (%)</v>
+        <v>Eingabe (%)</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Input (%)</v>
+        <v>Model fit — degree {deg}, {n} points</v>
       </c>
       <c r="B149" t="str">
-        <v>Eingabe (%)</v>
+        <v>Modellanpassung — Grad {deg}, {n} Punkte</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Model fit — degree {deg}, {n} points</v>
+        <v>↻ Regenerate</v>
       </c>
       <c r="B150" t="str">
-        <v>Modellanpassung — Grad {deg}, {n} Punkte</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="str">
-        <v>↻ Regenerate</v>
-      </c>
-      <c r="B151" t="str">
         <v>↻ Neu erstellen</v>
+      </c>
+    </row>
+    <row r="151" xml:space="preserve">
+      <c r="A151" t="str" xml:space="preserve">
+        <v xml:space="preserve">Input
+colorant</v>
+      </c>
+      <c r="B151" t="str" xml:space="preserve">
+        <v xml:space="preserve">Eingabe
+Farbmittel</v>
       </c>
     </row>
     <row r="152" xml:space="preserve">
       <c r="A152" t="str" xml:space="preserve">
-        <v xml:space="preserve">Input
-colorant</v>
-      </c>
-      <c r="B152" t="str" xml:space="preserve">
-        <v xml:space="preserve">Eingabe
-Farbmittel</v>
-      </c>
-    </row>
-    <row r="153" xml:space="preserve">
-      <c r="A153" t="str" xml:space="preserve">
         <v xml:space="preserve">Nearest
 in dataset</v>
       </c>
-      <c r="B153" t="str" xml:space="preserve">
+      <c r="B152" t="str" xml:space="preserve">
         <v xml:space="preserve">Nächster
 im Datensatz</v>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>Model</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Modell</v>
+      </c>
+    </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>Model</v>
+        <v>Computing…</v>
       </c>
       <c r="B154" t="str">
-        <v>Modell</v>
+        <v>Berechnung…</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>Computing…</v>
+        <v>Calculating tone values…</v>
       </c>
       <c r="B155" t="str">
-        <v>Berechnung…</v>
+        <v>Calculating tone values…</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>Calculating tone values…</v>
+        <v>Estimating model…</v>
       </c>
       <c r="B156" t="str">
-        <v>Calculating tone values…</v>
+        <v>Estimating model…</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>Estimating model…</v>
+        <v>Building 3D gamut…</v>
       </c>
       <c r="B157" t="str">
-        <v>Estimating model…</v>
+        <v>Building 3D gamut…</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>Building 3D gamut…</v>
+        <v>Computing 2D slice…</v>
       </c>
       <c r="B158" t="str">
-        <v>Building 3D gamut…</v>
+        <v>Computing 2D slice…</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>Computing 2D slice…</v>
+        <v>Rendering…</v>
       </c>
       <c r="B159" t="str">
-        <v>Computing 2D slice…</v>
+        <v>Rendering…</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>Rendering…</v>
+        <v>Model fit failed: {msg}</v>
       </c>
       <c r="B160" t="str">
-        <v>Rendering…</v>
+        <v>Modellanpassung fehlgeschlagen: {msg}</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>Model fit failed: {msg}</v>
+        <v>Retry</v>
       </c>
       <c r="B161" t="str">
-        <v>Modellanpassung fehlgeschlagen: {msg}</v>
+        <v>Wiederholen</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>Retry</v>
+        <v>Click on L*a*b* color to display spectral graph.</v>
       </c>
       <c r="B162" t="str">
-        <v>Wiederholen</v>
+        <v>Auf L*a*b*-Farbe klicken für Spektraldiagramm.</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>Click on L*a*b* color to display spectral graph.</v>
+        <v>Scroll to top</v>
       </c>
       <c r="B163" t="str">
-        <v>Auf L*a*b*-Farbe klicken für Spektraldiagramm.</v>
+        <v>Nach oben</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>Scroll to top</v>
+        <v>Top</v>
       </c>
       <c r="B164" t="str">
-        <v>Nach oben</v>
+        <v>Oben</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>Top</v>
+        <v>Help</v>
       </c>
       <c r="B165" t="str">
-        <v>Oben</v>
+        <v>Hilfe</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>Help</v>
+        <v>About CharData</v>
       </c>
       <c r="B166" t="str">
-        <v>Hilfe</v>
+        <v>Über CharData</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>About CharData</v>
+        <v>Support on Ko-fi</v>
       </c>
       <c r="B167" t="str">
-        <v>Über CharData</v>
+        <v>Ko-fi unterstützen</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>Support on Ko-fi</v>
+        <v>Buy me a coffee</v>
       </c>
       <c r="B168" t="str">
-        <v>Ko-fi unterstützen</v>
+        <v>Kauf mir einen Kaffee</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>Buy me a coffee</v>
+        <v>Reflectance</v>
       </c>
       <c r="B169" t="str">
-        <v>Kauf mir einen Kaffee</v>
+        <v>Reflexionsgrad</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>Reflectance</v>
+        <v>CharData is free for the color community. If it helps you, a small Ko-fi donation helps keep it running.</v>
       </c>
       <c r="B170" t="str">
-        <v>Reflexionsgrad</v>
+        <v>CharData ist für die Farbgemeinschaft kostenlos. Eine kleine Ko-fi-Spende hilft, den Dienst am Laufen zu halten.</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>CharData is free for the color community. If it helps you, a small Ko-fi donation helps keep it running.</v>
+        <v>Characterization data</v>
       </c>
       <c r="B171" t="str">
-        <v>CharData ist für die Farbgemeinschaft kostenlos. Eine kleine Ko-fi-Spende hilft, den Dienst am Laufen zu halten.</v>
+        <v>Charakterisierungsdaten</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>Characterization data</v>
+        <v>ICC Profiles</v>
       </c>
       <c r="B172" t="str">
-        <v>Charakterisierungsdaten</v>
+        <v>ICC-Profile</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>ICC Profiles</v>
+        <v>No characterization datasets loaded</v>
       </c>
       <c r="B173" t="str">
-        <v>ICC-Profile</v>
+        <v>Keine Charakterisierungsdaten geladen</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>No characterization datasets loaded</v>
+        <v>No ICC profiles loaded</v>
       </c>
       <c r="B174" t="str">
-        <v>Keine Charakterisierungsdaten geladen</v>
+        <v>Keine ICC-Profile geladen</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>No ICC profiles loaded</v>
+        <v>Characterization dataset</v>
       </c>
       <c r="B175" t="str">
-        <v>Keine ICC-Profile geladen</v>
+        <v>Charakterisierungsdatensatz</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>Characterization dataset</v>
+        <v>ICC Profile</v>
       </c>
       <c r="B176" t="str">
-        <v>Charakterisierungsdatensatz</v>
+        <v>ICC-Profil</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>ICC Profile</v>
+        <v>Not a valid ICC profile (header magic missing).</v>
       </c>
       <c r="B177" t="str">
-        <v>ICC-Profil</v>
+        <v>Kein gültiges ICC-Profil (Header-Signatur fehlt).</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>Not a valid ICC profile (header magic missing).</v>
+        <v>Standard datasets</v>
       </c>
       <c r="B178" t="str">
-        <v>Kein gültiges ICC-Profil (Header-Signatur fehlt).</v>
+        <v>Standarddatensätze</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>Standard datasets</v>
+        <v>Loading…</v>
       </c>
       <c r="B179" t="str">
-        <v>Standarddatensätze</v>
+        <v>Wird geladen…</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>Loading…</v>
+        <v>Failed to load list</v>
       </c>
       <c r="B180" t="str">
-        <v>Wird geladen…</v>
+        <v>Liste konnte nicht geladen werden</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>Failed to load list</v>
+        <v>Thickness:</v>
       </c>
       <c r="B181" t="str">
-        <v>Liste konnte nicht geladen werden</v>
+        <v>Dicke:</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>Thickness:</v>
+        <v>Fall-off:</v>
       </c>
       <c r="B182" t="str">
-        <v>Dicke:</v>
+        <v>Übergang:</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>Fall-off:</v>
+        <v>Hard</v>
       </c>
       <c r="B183" t="str">
-        <v>Übergang:</v>
+        <v>Hart</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>Hard</v>
+        <v>Soft</v>
       </c>
       <c r="B184" t="str">
-        <v>Hart</v>
+        <v>Weich</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>Soft</v>
+        <v>G7 validation is not available for ICC profiles.</v>
       </c>
       <c r="B185" t="str">
-        <v>Weich</v>
+        <v>G7-Validierung ist für ICC-Profile nicht verfügbar.</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>G7 validation is not available for ICC profiles.</v>
+        <v>ICC vs ICC comparison requires identical colorant lists. Profile A: {a}. Profile B: {b}.</v>
       </c>
       <c r="B186" t="str">
-        <v>G7-Validierung ist für ICC-Profile nicht verfügbar.</v>
+        <v>ICC-zu-ICC-Vergleich erfordert identische Farbmittellisten. Profil A: {a}. Profil B: {b}.</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>ICC vs ICC comparison requires identical colorant lists. Profile A: {a}. Profile B: {b}.</v>
+        <v>Dataset B does not contain colorants matching ICC profile A.</v>
       </c>
       <c r="B187" t="str">
-        <v>ICC-zu-ICC-Vergleich erfordert identische Farbmittellisten. Profil A: {a}. Profil B: {b}.</v>
+        <v>Datensatz B enthält keine Farbmittel, die zum ICC-Profil A passen.</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>Dataset B does not contain colorants matching ICC profile A.</v>
+        <v>Dataset A does not contain colorants matching ICC profile B.</v>
       </c>
       <c r="B188" t="str">
-        <v>Datensatz B enthält keine Farbmittel, die zum ICC-Profil A passen.</v>
+        <v>Datensatz A enthält keine Farbmittel, die zum ICC-Profil B passen.</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>Dataset A does not contain colorants matching ICC profile B.</v>
+        <v>Header</v>
       </c>
       <c r="B189" t="str">
-        <v>Datensatz A enthält keine Farbmittel, die zum ICC-Profil B passen.</v>
+        <v>Header</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>Header</v>
+        <v>Tags</v>
       </c>
       <c r="B190" t="str">
-        <v>Header</v>
+        <v>Tags</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>Tags</v>
+        <v>Loading ICC viewer…</v>
       </c>
       <c r="B191" t="str">
-        <v>Tags</v>
+        <v>ICC-Viewer wird geladen…</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>Loading ICC viewer…</v>
+        <v>Launch editor</v>
       </c>
       <c r="B192" t="str">
-        <v>ICC-Viewer wird geladen…</v>
+        <v>Editor öffnen</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>Launch editor</v>
+        <v>All data stays local to browser</v>
       </c>
       <c r="B193" t="str">
-        <v>Editor öffnen</v>
+        <v>Alle Daten bleiben lokal im Browser</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>All data stays local to browser</v>
+        <v>Free browser-resident online tool</v>
       </c>
       <c r="B194" t="str">
-        <v>Alle Daten bleiben lokal im Browser</v>
+        <v>Kostenloses Online-Tool, das im Browser läuft</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>Free browser-resident online tool</v>
+        <v>Image</v>
       </c>
       <c r="B195" t="str">
-        <v>Kostenloses Online-Tool, das im Browser läuft</v>
+        <v>Bild</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>Image</v>
+        <v>Load Image</v>
       </c>
       <c r="B196" t="str">
-        <v>Bild</v>
+        <v>Bild laden</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>Load Image</v>
+        <v>Bind image to dataset</v>
       </c>
       <c r="B197" t="str">
-        <v>Bild laden</v>
+        <v>Bild mit Datensatz verknüpfen</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>Bind image to dataset</v>
+        <v>Remove image</v>
       </c>
       <c r="B198" t="str">
-        <v>Bild mit Datensatz verknüpfen</v>
+        <v>Bild entfernen</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>Remove image</v>
+        <v>Image color space: {cs} {src}</v>
       </c>
       <c r="B199" t="str">
-        <v>Bild entfernen</v>
+        <v>Bildfarbraum: {cs} {src}</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>Image color space: {cs} {src}</v>
+        <v>Bound to {name} — {n} points</v>
       </c>
       <c r="B200" t="str">
-        <v>Bildfarbraum: {cs} {src}</v>
+        <v>Verknüpft mit {name} — {n} Punkte</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>Bound to {name} — {n} points</v>
+        <v>Lab image — {n} points</v>
       </c>
       <c r="B201" t="str">
-        <v>Verknüpft mit {name} — {n} Punkte</v>
+        <v>Lab-Bild — {n} Punkte</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>Lab image — {n} points</v>
+        <v>Cannot bind: image is {img} but Dataset {slot} is {family}.</v>
       </c>
       <c r="B202" t="str">
-        <v>Lab-Bild — {n} Punkte</v>
+        <v>Verknüpfung nicht möglich: Bild ist {img}, aber Datensatz {slot} ist {family}.</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>Cannot bind: image is {img} but Dataset {slot} is {family}.</v>
+        <v>Unsupported image format. Use PNG, JPEG, TIFF, BMP, GIF, or PDF.</v>
       </c>
       <c r="B203" t="str">
-        <v>Verknüpfung nicht möglich: Bild ist {img}, aber Datensatz {slot} ist {family}.</v>
+        <v>Bildformat nicht unterstützt. Bitte PNG, JPEG, TIFF, BMP, GIF oder PDF verwenden.</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>Unsupported image format. Use PNG, JPEG, TIFF, BMP, GIF, or PDF.</v>
+        <v>“{name}” is too large ({mb} MB). Maximum image size is {max} MB.</v>
       </c>
       <c r="B204" t="str">
-        <v>Bildformat nicht unterstützt. Bitte PNG, JPEG, TIFF, BMP, GIF oder PDF verwenden.</v>
+        <v>„{name}“ ist zu groß ({mb} MB). Maximale Bildgröße: {max} MB.</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>“{name}” is too large ({mb} MB). Maximum image size is {max} MB.</v>
+        <v>Embedded: {name}</v>
       </c>
       <c r="B205" t="str">
-        <v>„{name}“ ist zu groß ({mb} MB). Maximale Bildgröße: {max} MB.</v>
+        <v>Eingebettet: {name}</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>Embedded: {name}</v>
+        <v>Decoding image…</v>
       </c>
       <c r="B206" t="str">
-        <v>Eingebettet: {name}</v>
+        <v>Bild wird dekodiert …</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>Decoding image…</v>
+        <v>Image file is too small or corrupt.</v>
       </c>
       <c r="B207" t="str">
-        <v>Bild wird dekodiert …</v>
+        <v>Bilddatei ist zu klein oder beschädigt.</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>Image file is too small or corrupt.</v>
+        <v>TIFF decoder library failed to load.</v>
       </c>
       <c r="B208" t="str">
-        <v>Bilddatei ist zu klein oder beschädigt.</v>
+        <v>TIFF-Decoder-Bibliothek konnte nicht geladen werden.</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>TIFF decoder library failed to load.</v>
+        <v>Selected dataset model is still loading — try again in a moment.</v>
       </c>
       <c r="B209" t="str">
-        <v>TIFF-Decoder-Bibliothek konnte nicht geladen werden.</v>
+        <v>Das Modell des gewählten Datensatzes wird noch geladen — bitte gleich erneut versuchen.</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>Selected dataset model is still loading — try again in a moment.</v>
+        <v>Image decode failed.</v>
       </c>
       <c r="B210" t="str">
-        <v>Das Modell des gewählten Datensatzes wird noch geladen — bitte gleich erneut versuchen.</v>
+        <v>Bilddekodierung fehlgeschlagen.</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>Image decode failed.</v>
+        <v>No color dataset loaded.</v>
       </c>
       <c r="B211" t="str">
-        <v>Bilddekodierung fehlgeschlagen.</v>
+        <v>Kein Farbdatensatz geladen.</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>No color dataset loaded.</v>
+        <v>Embedded profile is no longer available.</v>
       </c>
       <c r="B212" t="str">
-        <v>Kein Farbdatensatz geladen.</v>
+        <v>Eingebettetes Profil ist nicht mehr verfügbar.</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>Embedded profile is no longer available.</v>
+        <v>(from embedded ICC)</v>
       </c>
       <c r="B213" t="str">
-        <v>Eingebettetes Profil ist nicht mehr verfügbar.</v>
+        <v>(aus eingebettetem ICC)</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>(from embedded ICC)</v>
+        <v>(TIFF Lab)</v>
       </c>
       <c r="B214" t="str">
-        <v>(aus eingebettetem ICC)</v>
+        <v>(TIFF Lab)</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>(TIFF Lab)</v>
+        <v>(inferred from channels)</v>
       </c>
       <c r="B215" t="str">
-        <v>(TIFF Lab)</v>
+        <v>(aus Kanälen abgeleitet)</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>(inferred from channels)</v>
+        <v>{n} representative points after binning + dedupe</v>
       </c>
       <c r="B216" t="str">
-        <v>(aus Kanälen abgeleitet)</v>
+        <v>{n} repräsentative Punkte nach Binning + Deduplizierung</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>{n} representative points after binning + dedupe</v>
+        <v>PDF support is limited to single-image Photoshop PDFs. Save as TIFF, JPEG, PNG, BMP, or GIF for other PDF content.</v>
       </c>
       <c r="B217" t="str">
-        <v>{n} repräsentative Punkte nach Binning + Deduplizierung</v>
+        <v>PDF-Unterstützung beschränkt sich auf Einzelbild-Photoshop-PDFs. Für andere PDF-Inhalte als TIFF, JPEG, PNG, BMP oder GIF speichern.</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>PDF support is limited to single-image Photoshop PDFs. Save as TIFF, JPEG, PNG, BMP, or GIF for other PDF content.</v>
+        <v>Encrypted PDFs are not supported.</v>
       </c>
       <c r="B218" t="str">
-        <v>PDF-Unterstützung beschränkt sich auf Einzelbild-Photoshop-PDFs. Für andere PDF-Inhalte als TIFF, JPEG, PNG, BMP oder GIF speichern.</v>
+        <v>Verschlüsselte PDFs werden nicht unterstützt.</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>Encrypted PDFs are not supported.</v>
+        <v>Only single-page Photoshop PDFs are supported.</v>
       </c>
       <c r="B219" t="str">
-        <v>Verschlüsselte PDFs werden nicht unterstützt.</v>
+        <v>Nur einseitige Photoshop-PDFs werden unterstützt.</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
-        <v>Only single-page Photoshop PDFs are supported.</v>
+        <v>PDF structure could not be parsed.</v>
       </c>
       <c r="B220" t="str">
-        <v>Nur einseitige Photoshop-PDFs werden unterstützt.</v>
+        <v>PDF-Struktur konnte nicht gelesen werden.</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>PDF structure could not be parsed.</v>
+        <v>No image found inside the PDF.</v>
       </c>
       <c r="B221" t="str">
-        <v>PDF-Struktur konnte nicht gelesen werden.</v>
+        <v>Im PDF wurde kein Bild gefunden.</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
-        <v>No image found inside the PDF.</v>
+        <v>PDF colour space is not supported. Use Gray, RGB, CMYK, or an ICC-based profile.</v>
       </c>
       <c r="B222" t="str">
-        <v>Im PDF wurde kein Bild gefunden.</v>
+        <v>PDF-Farbraum nicht unterstützt. Verwenden Sie Grau, RGB, CMYK oder ein ICC-basiertes Profil.</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>PDF colour space is not supported. Use Gray, RGB, CMYK, or an ICC-based profile.</v>
+        <v>PDF image filter is not supported. Re-save the PDF with JPEG or ZIP compression.</v>
       </c>
       <c r="B223" t="str">
-        <v>PDF-Farbraum nicht unterstützt. Verwenden Sie Grau, RGB, CMYK oder ein ICC-basiertes Profil.</v>
+        <v>PDF-Bildfilter nicht unterstützt. PDF mit JPEG- oder ZIP-Komprimierung erneut speichern.</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>PDF image filter is not supported. Re-save the PDF with JPEG or ZIP compression.</v>
+        <v>Close file select</v>
       </c>
       <c r="B224" t="str">
-        <v>PDF-Bildfilter nicht unterstützt. PDF mit JPEG- oder ZIP-Komprimierung erneut speichern.</v>
+        <v>Dateiauswahl schließen</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>Close file select</v>
+        <v>Drag to resize</v>
       </c>
       <c r="B225" t="str">
-        <v>Dateiauswahl schließen</v>
+        <v>Ziehen zum Ändern der Größe</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>Drag to resize</v>
+        <v>Contact</v>
       </c>
       <c r="B226" t="str">
-        <v>Ziehen zum Ändern der Größe</v>
+        <v>Kontakt</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
-        <v>Contact</v>
+        <v>Remove file</v>
       </c>
       <c r="B227" t="str">
-        <v>Kontakt</v>
+        <v>Datei entfernen</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
-        <v>Remove file</v>
+        <v>Rendering intent:</v>
       </c>
       <c r="B228" t="str">
-        <v>Datei entfernen</v>
+        <v>Rendering-Intent:</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
-        <v>Rendering intent:</v>
+        <v>Perceptual</v>
       </c>
       <c r="B229" t="str">
-        <v>Rendering-Intent:</v>
+        <v>Perzeptiv</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
-        <v>Perceptual</v>
+        <v>Relative Colorimetric</v>
       </c>
       <c r="B230" t="str">
-        <v>Perzeptiv</v>
+        <v>Relativ farbmetrisch</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
-        <v>Relative Colorimetric</v>
+        <v>Saturation</v>
       </c>
       <c r="B231" t="str">
-        <v>Relativ farbmetrisch</v>
+        <v>Sättigung</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
-        <v>Saturation</v>
+        <v>Absolute Colorimetric</v>
       </c>
       <c r="B232" t="str">
-        <v>Sättigung</v>
+        <v>Absolut farbmetrisch</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
-        <v>Absolute Colorimetric</v>
+        <v>System default ({lang})</v>
       </c>
       <c r="B233" t="str">
-        <v>Absolut farbmetrisch</v>
+        <v>Systemstandard ({lang})</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>System default ({lang})</v>
+        <v>ICC load error: {msg}</v>
       </c>
       <c r="B234" t="str">
-        <v>Systemstandard ({lang})</v>
+        <v>ICC-Ladefehler: {msg}</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>ICC load error: {msg}</v>
+        <v>Could not parse ICC profile: {msg}</v>
       </c>
       <c r="B235" t="str">
-        <v>ICC-Ladefehler: {msg}</v>
+        <v>ICC-Profil konnte nicht analysiert werden: {msg}</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>Could not parse ICC profile: {msg}</v>
+        <v>Popup blocked — allow popups for this site to launch the editor.</v>
       </c>
       <c r="B236" t="str">
-        <v>ICC-Profil konnte nicht analysiert werden: {msg}</v>
+        <v>Popup blockiert — bitte Popups für diese Seite zulassen, um den Editor zu starten.</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
-        <v>Popup blocked — allow popups for this site to launch the editor.</v>
+        <v>Failed to load {name}: {msg}</v>
       </c>
       <c r="B237" t="str">
-        <v>Popup blockiert — bitte Popups für diese Seite zulassen, um den Editor zu starten.</v>
+        <v>{name} konnte nicht geladen werden: {msg}</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
-        <v>Failed to load {name}: {msg}</v>
+        <v>Color space</v>
       </c>
       <c r="B238" t="str">
-        <v>{name} konnte nicht geladen werden: {msg}</v>
+        <v>Farbraum</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
-        <v>Color space</v>
+        <v>Device class</v>
       </c>
       <c r="B239" t="str">
-        <v>Farbraum</v>
+        <v>Geräteklasse</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
-        <v>Device class</v>
+        <v>Colorants</v>
       </c>
       <c r="B240" t="str">
-        <v>Geräteklasse</v>
+        <v>Farbmittel</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
-        <v>Colorants</v>
+        <v>Rendering intents</v>
       </c>
       <c r="B241" t="str">
-        <v>Farbmittel</v>
+        <v>Rendering-Intents</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
-        <v>Rendering intents</v>
+        <v>ICC A2B Evaluation</v>
       </c>
       <c r="B242" t="str">
-        <v>Rendering-Intents</v>
+        <v>ICC-A2B-Auswertung</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
-        <v>ICC A2B Evaluation</v>
+        <v>ICC Output</v>
       </c>
       <c r="B243" t="str">
-        <v>ICC-A2B-Auswertung</v>
+        <v>ICC-Ausgabe</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
-        <v>ICC Output</v>
+        <v>Image detail</v>
       </c>
       <c r="B244" t="str">
-        <v>ICC-Ausgabe</v>
+        <v>Bilddetailgrad</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
-        <v>Image detail</v>
+        <v>Coarse</v>
       </c>
       <c r="B245" t="str">
-        <v>Bilddetailgrad</v>
+        <v>Grob</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
-        <v>Coarse</v>
+        <v>Standard</v>
       </c>
       <c r="B246" t="str">
-        <v>Grob</v>
+        <v>Standard</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
-        <v>Standard</v>
+        <v>Fine</v>
       </c>
       <c r="B247" t="str">
-        <v>Standard</v>
+        <v>Fein</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
-        <v>Fine</v>
+        <v>Subscribe</v>
       </c>
       <c r="B248" t="str">
-        <v>Fein</v>
+        <v>Abonnieren</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
-        <v>Subscribe</v>
+        <v>Get notified about new chardata releases</v>
       </c>
       <c r="B249" t="str">
-        <v>Abonnieren</v>
+        <v>Bei neuen chardata-Releases benachrichtigt werden</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
-        <v>Get notified about new chardata releases</v>
+        <v>Get notified about new releases</v>
       </c>
       <c r="B250" t="str">
-        <v>Bei neuen chardata-Releases benachrichtigt werden</v>
+        <v>Bei neuen Releases benachrichtigt werden</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
-        <v>Get notified about new releases</v>
+        <v>Close</v>
       </c>
       <c r="B251" t="str">
-        <v>Bei neuen Releases benachrichtigt werden</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
-        <v>Close</v>
+        <v>We’ll email you when a new major or minor chardata release ships. Patch releases are skipped. Your address is reviewed manually before being added.</v>
       </c>
       <c r="B252" t="str">
-        <v>Schließen</v>
+        <v>Wir benachrichtigen Sie per E-Mail, sobald ein neues Major- oder Minor-Release von chardata erscheint. Patch-Releases werden übersprungen. Ihre Adresse wird manuell geprüft, bevor sie aufgenommen wird.</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
-        <v>We’ll email you when a new major or minor chardata release ships. Patch releases are skipped. Your address is reviewed manually before being added.</v>
+        <v>Email address</v>
       </c>
       <c r="B253" t="str">
-        <v>Wir benachrichtigen Sie per E-Mail, sobald ein neues Major- oder Minor-Release von chardata erscheint. Patch-Releases werden übersprungen. Ihre Adresse wird manuell geprüft, bevor sie aufgenommen wird.</v>
+        <v>E-Mail-Adresse</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
-        <v>Email address</v>
+        <v>you@example.com</v>
       </c>
       <c r="B254" t="str">
-        <v>E-Mail-Adresse</v>
+        <v>sie@example.com</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
-        <v>you@example.com</v>
+        <v>How will you use chardata?</v>
       </c>
       <c r="B255" t="str">
-        <v>sie@example.com</v>
+        <v>Wofür werden Sie chardata nutzen?</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
-        <v>How will you use chardata?</v>
+        <v>(optional)</v>
       </c>
       <c r="B256" t="str">
-        <v>Wofür werden Sie chardata nutzen?</v>
+        <v>(optional)</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
-        <v>(optional)</v>
+        <v>e.g. evaluating ICC profiles for press calibration</v>
       </c>
       <c r="B257" t="str">
-        <v>(optional)</v>
+        <v>z. B. ICC-Profile für Druckkalibrierung evaluieren</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>e.g. evaluating ICC profiles for press calibration</v>
+        <v>I agree to receive emails about chardata releases. I can unsubscribe at any time.</v>
       </c>
       <c r="B258" t="str">
-        <v>z. B. ICC-Profile für Druckkalibrierung evaluieren</v>
+        <v>Ich willige ein, E-Mails über chardata-Releases zu erhalten. Ich kann mich jederzeit abmelden.</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>I agree to receive emails about chardata releases. I can unsubscribe at any time.</v>
+        <v>Subscribe</v>
       </c>
       <c r="B259" t="str">
-        <v>Ich willige ein, E-Mails über chardata-Releases zu erhalten. Ich kann mich jederzeit abmelden.</v>
+        <v>Abonnieren</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>Subscribe</v>
+        <v>Thanks — we’ll be in touch.</v>
       </c>
       <c r="B260" t="str">
-        <v>Abonnieren</v>
+        <v>Danke — wir melden uns.</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>Thanks — we’ll be in touch.</v>
+        <v>Once approved you’ll receive a welcome email. After that, you’ll only hear from us when a new chardata release ships.</v>
       </c>
       <c r="B261" t="str">
-        <v>Danke — wir melden uns.</v>
+        <v>Nach Freigabe erhalten Sie eine Willkommens-E-Mail. Danach hören Sie nur dann von uns, wenn ein neues chardata-Release erscheint.</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>Once approved you’ll receive a welcome email. After that, you’ll only hear from us when a new chardata release ships.</v>
+        <v>Close</v>
       </c>
       <c r="B262" t="str">
-        <v>Nach Freigabe erhalten Sie eine Willkommens-E-Mail. Danach hören Sie nur dann von uns, wenn ein neues chardata-Release erscheint.</v>
+        <v>Schließen</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>Close</v>
+        <v>Privacy notice</v>
       </c>
       <c r="B263" t="str">
-        <v>Schließen</v>
+        <v>Datenschutzhinweis</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>Privacy notice</v>
+        <v>Measurement-only data (no device colorants): 3D and 2D-slice point cloud, data table, and label-matched compare are available; gamut shell, extract, tone value, estimate, and validation are disabled.</v>
       </c>
       <c r="B264" t="str">
-        <v>Datenschutzhinweis</v>
+        <v>Nur Messdaten (keine Gerätefarbmittel): 3D- und 2D-Schnitt-Punktwolke, Datentabelle und etikettenbasierter Vergleich verfügbar; Gamut-Hülle, Extrahieren, Tonwert, Schätzung und Validierung deaktiviert.</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>Measurement-only data (no device colorants): 3D and 2D-slice point cloud, data table, and label-matched compare are available; gamut shell, extract, tone value, estimate, and validation are disabled.</v>
+        <v>Sample</v>
       </c>
       <c r="B265" t="str">
-        <v>Nur Messdaten (keine Gerätefarbmittel): 3D- und 2D-Schnitt-Punktwolke, Datentabelle und etikettenbasierter Vergleich verfügbar; Gamut-Hülle, Extrahieren, Tonwert, Schätzung und Validierung deaktiviert.</v>
+        <v>Probe</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>Sample</v>
+        <v>CxF file is not well-formed XML.</v>
       </c>
       <c r="B266" t="str">
-        <v>Probe</v>
+        <v>CxF-Datei ist kein wohlgeformtes XML.</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>CxF file is not well-formed XML.</v>
+        <v>CxF file contains no colour objects.</v>
       </c>
       <c r="B267" t="str">
-        <v>CxF-Datei ist kein wohlgeformtes XML.</v>
+        <v>CxF-Datei enthält keine Farbobjekte.</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>CxF file contains no colour objects.</v>
+        <v>CxF file contains no CIELab or spectral colour values.</v>
       </c>
       <c r="B268" t="str">
-        <v>CxF-Datei enthält keine Farbobjekte.</v>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="str">
-        <v>CxF file contains no CIELab or spectral colour values.</v>
-      </c>
-      <c r="B269" t="str">
         <v>CxF-Datei enthält keine CIELab- oder Spektralfarbwerte.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B269"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B268"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1.9.1: CxF/X-4 (ISO 17972-4) spot ink characterisation support
parseCxF now recognises the SpotInkCharacterisation custom resource:
tint levels become a device colorant named from SpotInkName, plus a
PROCESS_BLACK 0/100 backing colorant when both backgrounds are present.
Conformance level (CxF/X-4 / X-4a / X-4b) is detected and shown as the
file type label. Tables, plots, Tone Value, Extract and Compare all
work as for any characterisation data; model-based features (gamut
shell, Estimate) are gated off via state.noModel since 1-2-colorant
tint ramps can't support the polynomial model.

Also: ReflectanceSpectrum StartWL now falls back to the referenced
ColorSpecification's WavelengthRange (X-4 files only declare it there);
the CxF type label and file-panel notices survive a live language
switch; new cxfx4_notice i18n key in all 12 locales + xlsx sheets.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B308"/>
+  <dimension ref="A1:B309"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2871,9 +2871,17 @@
         <v>Daten</v>
       </c>
     </row>
+    <row r="309">
+      <c r="A309" t="str">
+        <v>Spot ink characterisation (CxF/X-4): tint levels are loaded as device colorant values; gamut shell, estimate, and model generation are disabled.</v>
+      </c>
+      <c r="B309" t="str">
+        <v>Sonderfarben-Charakterisierung (CxF/X-4): Tonwertstufen werden als Gerätefarbmittelwerte geladen; Gamut-Hülle, Schätzung und Modellerzeugung deaktiviert.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B308"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B309"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1.10.0: resizable plot height (aspect ratio) + Gamut Slice scroll-wheel zoom
3D Plot and Gamut Slice now have a draggable bottom-edge handle (the same
3-dots grip + hover/dragging highlight as the File Select pane) that changes
the plot height. The chosen height is sticky per plot (localStorage
plot3dHeight / sliceHeight). Auto-scaling of the data is untouched — only the
canvas box changes.

Gamut Slice also gains mouse scroll-wheel zoom (rescales the auto-scaled range
about its centre via Plotly.relayout, no WASM rebuild) plus a Reset zoom
control. New reset_zoom string localized across all 12 in-page locales and the
9 Eng-*.xlsx spreadsheets.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B309"/>
+  <dimension ref="A1:B310"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2879,9 +2879,17 @@
         <v>Sonderfarben-Charakterisierung (CxF/X-4): Tonwertstufen werden als Gerätefarbmittelwerte geladen; Gamut-Hülle, Schätzung und Modellerzeugung deaktiviert.</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="str">
+        <v>Reset zoom</v>
+      </c>
+      <c r="B310" t="str">
+        <v>Zoom zurücksetzen</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B309"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B310"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1.14.0: Comparison Statistics tab + ΔE distribution histogram
Move the bulk ΔE statistics (mean / min / max / std dev) into their own
collapsible "Comparison Statistics" section in Compare mode (closed by default),
and add a ΔE distribution histogram below the numbers: relative-frequency bars
(left axis) plus a cumulative-frequency line (right axis), built from the same
matched-patch ΔE list and the ΔE method selected in Settings.

A "Horizontal scale" switch toggles the ΔE axis between Integer ΔE bins (default)
and Auto-scale with a user-specified bin count (1–100); the choice persists.
Works across all Compare combinations (data/data, data/ICC, ICC/ICC), is
dark-mode aware, and is localized across all 12 languages (dict + xlsx). User
guide updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B320"/>
+  <dimension ref="A1:B327"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2967,9 +2967,65 @@
         <v>Gamut-Gitternetz anzeigen</v>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" t="str">
+        <v>Comparison Statistics</v>
+      </c>
+      <c r="B321" t="str">
+        <v>Vergleichsstatistik</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="str">
+        <v>Relative frequency</v>
+      </c>
+      <c r="B322" t="str">
+        <v>Relative Häufigkeit</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="str">
+        <v>Cumulative frequency</v>
+      </c>
+      <c r="B323" t="str">
+        <v>Kumulative Häufigkeit</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="str">
+        <v>Horizontal scale</v>
+      </c>
+      <c r="B324" t="str">
+        <v>Horizontale Skala</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="str">
+        <v>Integer ΔE</v>
+      </c>
+      <c r="B325" t="str">
+        <v>Ganzzahliges ΔE</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="str">
+        <v>Auto-scale</v>
+      </c>
+      <c r="B326" t="str">
+        <v>Auto-Skalierung</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="str">
+        <v>Bins</v>
+      </c>
+      <c r="B327" t="str">
+        <v>Klassen</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B320"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B327"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1.15.0: 3D plot rotation controls
Adds a Rotation group to the 3D plot's collapsible Controls panel:
- Mode: Turntable (default) / Orbit — same knob as Plotly's in-frame
  modebar rotation buttons, surfaced where it's easy to find.
- Drag rotate sensitivity (0.1-3, default 1) — scales click-and-drag orbit
  via the gl3d camera's rotateSpeed.
- Enable roll (horizontal scroll) on/off.
- Roll sensitivity (0.05-2, default 0.4) — an independent knob for the
  horizontal-scroll roll gesture.

Roll is now handled by a capture-phase wheel interceptor that owns every
horizontal-dominant wheel event, so its sensitivity is fully decoupled from
drag-orbit (rotateSpeed governs drag only). Vertical scroll still zooms.
All four settings persist in localStorage and re-sync to the controls on load.

i18n keys added across all 12 locales + translations/Eng-*.xlsx (0 drift).
MANUAL.md gains a Rotation subsection.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B327"/>
+  <dimension ref="A1:B334"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3023,9 +3023,65 @@
         <v>Klassen</v>
       </c>
     </row>
+    <row r="328">
+      <c r="A328" t="str">
+        <v>Rotation</v>
+      </c>
+      <c r="B328" t="str">
+        <v>Rotation</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="str">
+        <v>Mode:</v>
+      </c>
+      <c r="B329" t="str">
+        <v>Modus:</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="str">
+        <v>Turntable</v>
+      </c>
+      <c r="B330" t="str">
+        <v>Drehteller</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="str">
+        <v>Orbit</v>
+      </c>
+      <c r="B331" t="str">
+        <v>Orbit</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="str">
+        <v>Drag rotate sensitivity:</v>
+      </c>
+      <c r="B332" t="str">
+        <v>Empfindlichkeit Ziehen-Rotation:</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="str">
+        <v>Enable roll (horizontal scroll)</v>
+      </c>
+      <c r="B333" t="str">
+        <v>Rollen aktivieren (horizontales Scrollen)</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="str">
+        <v>Roll sensitivity:</v>
+      </c>
+      <c r="B334" t="str">
+        <v>Rollempfindlichkeit:</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B327"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B334"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Translations: sync xlsx with new QC + guide i18n strings
Adds the new guide (guide_*) and QC-feature strings (primaries/overprints,
near-neutral, comparison plot, percentiles, per-channel ΔE, duplicate
repeatability) across all locale spreadsheets, plus the previously-missing
image_err_too_big row. check-translations now reports zero drift.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014NduGJdN1Sp1KPX3KSjMPn
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B334"/>
+  <dimension ref="A1:B377"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3079,9 +3079,353 @@
         <v>Rollempfindlichkeit:</v>
       </c>
     </row>
+    <row r="335">
+      <c r="A335" t="str">
+        <v>Primaries &amp; Overprints</v>
+      </c>
+      <c r="B335" t="str">
+        <v>Primärfarben &amp; Überdrucke</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="str">
+        <v>Patch</v>
+      </c>
+      <c r="B336" t="str">
+        <v>Feld</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="str">
+        <v>Paper</v>
+      </c>
+      <c r="B337" t="str">
+        <v>Papier</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="str">
+        <v>Cyan</v>
+      </c>
+      <c r="B338" t="str">
+        <v>Cyan</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="str">
+        <v>Magenta</v>
+      </c>
+      <c r="B339" t="str">
+        <v>Magenta</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="str">
+        <v>Yellow</v>
+      </c>
+      <c r="B340" t="str">
+        <v>Gelb</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="str">
+        <v>Black</v>
+      </c>
+      <c r="B341" t="str">
+        <v>Schwarz</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="str">
+        <v>Red</v>
+      </c>
+      <c r="B342" t="str">
+        <v>Rot</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="str">
+        <v>Green</v>
+      </c>
+      <c r="B343" t="str">
+        <v>Grün</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="str">
+        <v>Blue</v>
+      </c>
+      <c r="B344" t="str">
+        <v>Blau</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="str">
+        <v>CMY</v>
+      </c>
+      <c r="B345" t="str">
+        <v>CMY</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="str">
+        <v>CMYK</v>
+      </c>
+      <c r="B346" t="str">
+        <v>CMYK</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="str">
+        <v>Found {n} duplicate measurements in the original dataset.</v>
+      </c>
+      <c r="B347" t="str">
+        <v>{n} doppelte Messungen im ursprünglichen Datensatz gefunden.</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="str">
+        <v>Found {n} duplicate measurements in the original dataset (repeatability ΔE mean {mean}, max {max}).</v>
+      </c>
+      <c r="B348" t="str">
+        <v>{n} doppelte Messungen im ursprünglichen Datensatz gefunden (Wiederholbarkeit ΔE Mittel {mean}, Max {max}).</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="str">
+        <v>Near-Neutral Survey</v>
+      </c>
+      <c r="B349" t="str">
+        <v>Quasi-Neutral-Analyse</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="str">
+        <v>Threshold (ΔE*ab)</v>
+      </c>
+      <c r="B350" t="str">
+        <v>Schwellenwert (ΔE*ab)</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="str">
+        <v>{near} of {total} patches within {thr} ΔE of neutral.</v>
+      </c>
+      <c r="B351" t="str">
+        <v>{near} von {total} Feldern liegen innerhalb von {thr} ΔE zum Neutral.</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="str">
+        <v>No patches within {thr} ΔE of neutral.</v>
+      </c>
+      <c r="B352" t="str">
+        <v>Keine Felder innerhalb von {thr} ΔE zum Neutral.</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="str">
+        <v>Distance from neutral (ΔE*ab)</v>
+      </c>
+      <c r="B353" t="str">
+        <v>Abstand zum Neutral (ΔE*ab)</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="str">
+        <v>Near-neutral</v>
+      </c>
+      <c r="B354" t="str">
+        <v>Quasi-neutral</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="str">
+        <v>Other patches</v>
+      </c>
+      <c r="B355" t="str">
+        <v>Andere Felder</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="str">
+        <v>Comparison Plot</v>
+      </c>
+      <c r="B356" t="str">
+        <v>Vergleichsdiagramm</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="str">
+        <v>P90 = {v}</v>
+      </c>
+      <c r="B357" t="str">
+        <v>P90 = {v}</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="str">
+        <v>Percentiles</v>
+      </c>
+      <c r="B358" t="str">
+        <v>Perzentile</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="str">
+        <v>Per-channel ΔE</v>
+      </c>
+      <c r="B359" t="str">
+        <v>ΔE pro Kanal</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="str">
+        <v>Included: patches using this ink (&gt;0). Excluded: patches without it. Only: this ink alone.</v>
+      </c>
+      <c r="B360" t="str">
+        <v>Enthalten: Felder mit dieser Farbe (&gt;0). Ausgeschlossen: Felder ohne sie. Nur: nur diese Farbe.</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="str">
+        <v>Included</v>
+      </c>
+      <c r="B361" t="str">
+        <v>Enthalten</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="str">
+        <v>Excluded</v>
+      </c>
+      <c r="B362" t="str">
+        <v>Ausgeschlossen</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="str">
+        <v>Only</v>
+      </c>
+      <c r="B363" t="str">
+        <v>Nur</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="str">
+        <v>N</v>
+      </c>
+      <c r="B364" t="str">
+        <v>N</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="str">
+        <v>P90</v>
+      </c>
+      <c r="B365" t="str">
+        <v>P90</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="str">
+        <v>P95</v>
+      </c>
+      <c r="B366" t="str">
+        <v>P95</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="str">
+        <v>Max</v>
+      </c>
+      <c r="B367" t="str">
+        <v>Max</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="str">
+        <v>User Guide</v>
+      </c>
+      <c r="B368" t="str">
+        <v>Benutzerhandbuch</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="str">
+        <v>Search the guide…</v>
+      </c>
+      <c r="B369" t="str">
+        <v>Handbuch durchsuchen…</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="str">
+        <v>Previous match</v>
+      </c>
+      <c r="B370" t="str">
+        <v>Vorheriger Treffer</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="str">
+        <v>Next match</v>
+      </c>
+      <c r="B371" t="str">
+        <v>Nächster Treffer</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="str">
+        <v>Open in a new tab</v>
+      </c>
+      <c r="B372" t="str">
+        <v>In neuem Tab öffnen</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="str">
+        <v>Loading the guide…</v>
+      </c>
+      <c r="B373" t="str">
+        <v>Handbuch wird geladen…</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="str">
+        <v>Couldn’t load the guide. Try opening it in a new tab.</v>
+      </c>
+      <c r="B374" t="str">
+        <v>Handbuch konnte nicht geladen werden. Versuchen Sie, es in einem neuen Tab zu öffnen.</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="str">
+        <v>No matches</v>
+      </c>
+      <c r="B375" t="str">
+        <v>Keine Treffer</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="str">
+        <v>{i}/{n}</v>
+      </c>
+      <c r="B376" t="str">
+        <v>{i}/{n}</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="str">
+        <v>Image is too large to process safely.</v>
+      </c>
+      <c r="B377" t="str">
+        <v>Bild ist zu groß, um sicher verarbeitet zu werden.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B334"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B377"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
1.17.0: L* Reversal analysis section
New Explore-mode collapsible (char data only) that checks each single-ink
tint ramp for L* reversals — steps where adding ink lightens instead of
darkening. Per-colorant L*-vs-ink% chart with red reversal-segment overlay, a
worst-first ranked table (colorant / ink range / ΔL*), and a persisted ΔL*
threshold. Works on measured ramps directly (covers CxF/X-4 spot inks); repeat
ink levels are averaged so repeatability scatter isn't misread. Localized across
12 locales + xlsx; documented in the user guide (§4.7).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MZHEB81USqdMVasHnkQYre
</commit_message>
<xml_diff>
--- a/translations/Eng-De.xlsx
+++ b/translations/Eng-De.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B377"/>
+  <dimension ref="A1:B386"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3423,9 +3423,81 @@
         <v>Bild ist zu groß, um sicher verarbeitet zu werden.</v>
       </c>
     </row>
+    <row r="378">
+      <c r="A378" t="str">
+        <v>L* Reversal</v>
+      </c>
+      <c r="B378" t="str">
+        <v>L*-Umkehr</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="str">
+        <v>Adding ink to a single-ink tint ramp should only darken it. Each measured ramp is checked; any step where L* rises is flagged as a reversal.</v>
+      </c>
+      <c r="B379" t="str">
+        <v>Mehr Farbe auf einer Einzelfarben-Tonrampe sollte diese nur abdunkeln. Jede gemessene Rampe wird geprüft; jeder Schritt, bei dem L* ansteigt, wird als Umkehr markiert.</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="str">
+        <v>Threshold (ΔL*)</v>
+      </c>
+      <c r="B380" t="str">
+        <v>Schwellenwert (ΔL*)</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="str">
+        <v>{n} reversal(s) across {cols} ink ramp(s).</v>
+      </c>
+      <c r="B381" t="str">
+        <v>{n} Umkehr(en) über {cols} Farbrampe(n).</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="str">
+        <v>No L* reversals — every ink ramp darkens monotonically.</v>
+      </c>
+      <c r="B382" t="str">
+        <v>Keine L*-Umkehr — jede Farbrampe dunkelt monoton ab.</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="str">
+        <v>L* reversal</v>
+      </c>
+      <c r="B383" t="str">
+        <v>L*-Umkehr</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="str">
+        <v>Ink %</v>
+      </c>
+      <c r="B384" t="str">
+        <v>Farbe %</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="str">
+        <v>Colorant</v>
+      </c>
+      <c r="B385" t="str">
+        <v>Farbmittel</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="str">
+        <v>Ink range</v>
+      </c>
+      <c r="B386" t="str">
+        <v>Farbbereich</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B377"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B386"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>